<commit_message>
HU-064: describe fecha o bloco 0, e Quote.Status ja tem valores em espanhol
</commit_message>
<xml_diff>
--- a/docs/hu064/HU064_Tarefas_Tecnicas.xlsx
+++ b/docs/hu064/HU064_Tarefas_Tecnicas.xlsx
@@ -116,7 +116,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">FEITO 18/08</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">OrderItem nao tem Discount padrao. Criar so depois que o T01 confirmar, e com o mesmo nome e tipo do padrao da cotizacion</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T01</t>
+          <t xml:space="preserve">Criar o campo de percentual. Confirmado que OrderItem nao tem Discount padrao. O valor ja cabe em TotalLineAmount e em UnitPrice, que sao gravaveis, o que falta e so o percentual</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -809,7 +804,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">CONFIRMADO, criar</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1003,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Avaliar Quote.Status antes de criar campo de autorizacao</t>
+          <t xml:space="preserve">Decidir o valor de Quote.Status para requiere autorizacion</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1023,12 +1018,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ver no T01 se ja ha valor que sirva para requiere autorizacion. Se a picklist for restrita, acrescentar valor proprio faz a funcionalidade padrao ver algo que nao conhece</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T01</t>
+          <t xml:space="preserve">A picklist nao e restrita e ja tem Draft, Approved, Rejected, Accepted, Denied, mais Pendiente, Pedido futuro e En transito. Definir com o negocio se Pendiente serve ou se entra valor novo, antes de criar checkbox proprio</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1045,148 +1035,148 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">T23</t>
+          <t xml:space="preserve">T22b</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Passo de validacao contra o piso</t>
+          <t xml:space="preserve">Levantar os valores em espanhol ja acrescentados a Quote.Status</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">ExpressionSet</t>
+          <t xml:space="preserve">Divida</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Passo final do pricing procedure</t>
+          <t xml:space="preserve">Quote.Status</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comparar desconto mais cashback contra o piso do nivel do usuario e marcar a condicao quando exceder</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T13, T21</t>
+          <t xml:space="preserve">Pendiente, Pedido futuro e En transito estao com o valor de API em espanhol, contra a convencao GRPQM, e dois deles sao conceito de pedido dentro do status da cotizacion. Levantar quem criou e para que antes de acrescentar mais um valor</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN4, Escenario 2</t>
+          <t xml:space="preserve">Convencao GRPQM</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">ACHADO 18/08</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">T24</t>
+          <t xml:space="preserve">T23</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Definir se a advertencia bloqueia</t>
+          <t xml:space="preserve">Passo de validacao contra o piso</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision</t>
+          <t xml:space="preserve">ExpressionSet</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passo final do pricing procedure</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Perguntar ao GrupoQ. O Escenario 3 diz que impede continuar ate a aprovacao. O Flujo 7 diz que nao bloqueia e que so o envio e a impressao ficam bloqueados. Sao comportamentos opostos no mesmo gatilho</t>
+          <t xml:space="preserve">Comparar desconto mais cashback contra o piso do nivel do usuario e marcar a condicao quando exceder</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T13, T21</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Escenario 3, Flujo 7</t>
+          <t xml:space="preserve">RN4, Escenario 2</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOQUEADO</t>
+          <t xml:space="preserve">A FAZER</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">T25</t>
+          <t xml:space="preserve">T24</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alerta sem expor o montante limite</t>
+          <t xml:space="preserve">Definir se a advertencia bloqueia</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">LWC ou Flow</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aviso na tela de cotizacion</t>
+          <t xml:space="preserve">Decision</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Informar apenas que o desconto excede o permitido para o rol. Em Autos e Motos nunca mostrar o montante limite</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T23</t>
+          <t xml:space="preserve">Perguntar ao GrupoQ. O Escenario 3 diz que impede continuar ate a aprovacao. O Flujo 7 diz que nao bloqueia e que so o envio e a impressao ficam bloqueados. Sao comportamentos opostos no mesmo gatilho</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN4</t>
+          <t xml:space="preserve">Escenario 3, Flujo 7</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">BLOQUEADO</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">T26</t>
+          <t xml:space="preserve">T25</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alerta de configuracao ausente ou inativa</t>
+          <t xml:space="preserve">Alerta sem expor o montante limite</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow</t>
+          <t xml:space="preserve">LWC ou Flow</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aviso na tela de cotizacion</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Se nao houver registro ativo para a combinacao de marca, modelo e sociedade, informar a condicao e impedir desconto abaixo do Precio Minimo de Asesor, sem assumir valor por defeito</t>
+          <t xml:space="preserve">Informar apenas que o desconto excede o permitido para o rol. Em Autos e Motos nunca mostrar o montante limite</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">T04</t>
+          <t xml:space="preserve">T23</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Escenarios 9 e 10</t>
+          <t xml:space="preserve">RN4</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1198,12 +1188,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">T27</t>
+          <t xml:space="preserve">T26</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alerta de cliente sem grupo ou canal</t>
+          <t xml:space="preserve">Alerta de configuracao ausente ou inativa</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1213,12 +1203,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Informar a ausencia do dado. O motor detecta ausencia, nao valida se a atribuicao esta correta</t>
+          <t xml:space="preserve">Se nao houver registro ativo para a combinacao de marca, modelo e sociedade, informar a condicao e impedir desconto abaixo do Precio Minimo de Asesor, sem assumir valor por defeito</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T04</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Escenario 21</t>
+          <t xml:space="preserve">Escenarios 9 e 10</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1230,12 +1225,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">T28</t>
+          <t xml:space="preserve">T27</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alerta de regra vencida</t>
+          <t xml:space="preserve">Alerta de cliente sem grupo ou canal</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1245,12 +1240,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Informar ao vendedor que a regra de desconto ou de preco esta vencida e seguir para a proxima regra vigente</t>
+          <t xml:space="preserve">Informar a ausencia do dado. O motor detecta ausencia, nao valida se a atribuicao esta correta</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Escenario 20</t>
+          <t xml:space="preserve">Escenario 21</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1262,140 +1257,130 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOCO 6</t>
+          <t xml:space="preserve">T28</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">REPUESTOS E PA</t>
+          <t xml:space="preserve">Alerta de regra vencida</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flow</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informar ao vendedor que a regra de desconto ou de preco esta vencida e seguir para a proxima regra vigente</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Escenario 20</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A FAZER</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">T29</t>
+          <t xml:space="preserve">BLOCO 6</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exibir o preco construido pelo SAP sem recalcular</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ApexClass</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SapMuleClient e tela de linhas</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mostrar o preco com as condicoes do esquema ZGQREF ja incorporadas. Salesforce nao recalcula nem persiste os codigos de condicao</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RN3, Escenario 13</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">REPUESTOS E PA</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">T30</t>
+          <t xml:space="preserve">T29</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resolver como o Salesforce sabe de ZRMA e ZREC</t>
+          <t xml:space="preserve">Exibir o preco construido pelo SAP sem recalcular</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision</t>
+          <t xml:space="preserve">ApexClass</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contrato da resposta do MuleSoft</t>
+          <t xml:space="preserve">SapMuleClient e tela de linhas</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pedir ao time de Mule uma bandeira na resposta. A RN3 diz que o Salesforce nao ramifica por codigo do SAP, mas a RN7 e a RN14 exigem comportamento diferente para ZRMA, que retira todos os descontos, e para ZREC, que soma</t>
+          <t xml:space="preserve">Mostrar o preco com as condicoes do esquema ZGQREF ja incorporadas. Salesforce nao recalcula nem persiste os codigos de condicao</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN3, RN7, RN14</t>
+          <t xml:space="preserve">RN3, Escenario 13</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOQUEADO</t>
+          <t xml:space="preserve">A FAZER</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">T31</t>
+          <t xml:space="preserve">T30</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Avaliar so o desconto manual, linha a linha</t>
+          <t xml:space="preserve">Resolver como o Salesforce sabe de ZRMA e ZREC</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">ExpressionSet</t>
+          <t xml:space="preserve">Decision</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Passo de validacao</t>
+          <t xml:space="preserve">Contrato da resposta do MuleSoft</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Avaliar cada linha de forma independente contra o rango do rol e marcar a condicao so na linha que excede</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T23</t>
+          <t xml:space="preserve">Pedir ao time de Mule uma bandeira na resposta. A RN3 diz que o Salesforce nao ramifica por codigo do SAP, mas a RN7 e a RN14 exigem comportamento diferente para ZRMA, que retira todos os descontos, e para ZREC, que soma</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Escenario 16</t>
+          <t xml:space="preserve">RN3, RN7, RN14</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">BLOQUEADO</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">T32</t>
+          <t xml:space="preserve">T31</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precedencia entre automatico e manual</t>
+          <t xml:space="preserve">Avaliar so o desconto manual, linha a linha</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1405,22 +1390,22 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Passo de precedencia</t>
+          <t xml:space="preserve">Passo de validacao</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Selecionar uma so regra, a de maior percentual, e descartar a outra. Nunca somar descontos</t>
+          <t xml:space="preserve">Avaliar cada linha de forma independente contra o rango do rol e marcar a condicao so na linha que excede</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">T31</t>
+          <t xml:space="preserve">T23</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN7, Escenarios 15 e 24</t>
+          <t xml:space="preserve">Escenario 16</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -1432,37 +1417,37 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">T33</t>
+          <t xml:space="preserve">T32</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Desconto de lealdade apenas informado</t>
+          <t xml:space="preserve">Precedencia entre automatico e manual</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">ApexClass</t>
+          <t xml:space="preserve">ExpressionSet</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tela de linhas</t>
+          <t xml:space="preserve">Passo de precedencia</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Informar a condicao, nao expor o desconto no documento comercial e nao avaliar contra o rango do rol nem enviar a aprovacao</t>
+          <t xml:space="preserve">Selecionar uma so regra, a de maior percentual, e descartar a outra. Nunca somar descontos</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">T29</t>
+          <t xml:space="preserve">T31</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN14, Escenario 25</t>
+          <t xml:space="preserve">RN7, Escenarios 15 e 24</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -1474,12 +1459,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">T34</t>
+          <t xml:space="preserve">T33</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reconsulta ao trocar o indicador fiscal</t>
+          <t xml:space="preserve">Desconto de lealdade apenas informado</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1489,12 +1474,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">RepuestosLineService</t>
+          <t xml:space="preserve">Tela de linhas</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Disparar reconsulta de todas as linhas ao SAP quando o indicador mudar em Repuestos. Em Autos disparar recalculo local</t>
+          <t xml:space="preserve">Informar a condicao, nao expor o desconto no documento comercial e nao avaliar contra o rango do rol nem enviar a aprovacao</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -1504,7 +1489,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve">FA-04, Escenario 15</t>
+          <t xml:space="preserve">RN14, Escenario 25</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -1516,37 +1501,37 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">T35</t>
+          <t xml:space="preserve">T34</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rodar o motor tambem sobre o pedido</t>
+          <t xml:space="preserve">Reconsulta ao trocar o indicador fiscal</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">ExpressionSet</t>
+          <t xml:space="preserve">ApexClass</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mesmo pricing procedure em Order</t>
+          <t xml:space="preserve">RepuestosLineService</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resolver o desconto direto no pedido, com a mesma configuracao, quando nao existir cotizacion previa</t>
+          <t xml:space="preserve">Disparar reconsulta de todas as linhas ao SAP quando o indicador mudar em Repuestos. Em Autos disparar recalculo local</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve">T18</t>
+          <t xml:space="preserve">T29</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Escenario 17</t>
+          <t xml:space="preserve">FA-04, Escenario 15</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -1558,12 +1543,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">T36</t>
+          <t xml:space="preserve">T35</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nao recalcular por condicao de pagamento, retencao ou moeda</t>
+          <t xml:space="preserve">Rodar o motor tambem sobre o pedido</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1573,22 +1558,22 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Passo de determinacao</t>
+          <t xml:space="preserve">Mesmo pricing procedure em Order</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conservar o desconto ja calculado quando mudarem esses tres. Nao sao criterios de determinacao</t>
+          <t xml:space="preserve">Resolver o desconto direto no pedido, com a mesma configuracao, quando nao existir cotizacion previa</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">T31</t>
+          <t xml:space="preserve">T18</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Escenario 18</t>
+          <t xml:space="preserve">Escenario 17</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -1600,86 +1585,81 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOCO 7</t>
+          <t xml:space="preserve">T36</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARGEM E RASTREABILIDADE</t>
+          <t xml:space="preserve">Nao recalcular por condicao de pagamento, retencao ou moeda</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ExpressionSet</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passo de determinacao</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conservar o desconto ja calculado quando mudarem esses tres. Nao sao criterios de determinacao</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T31</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Escenario 18</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A FAZER</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">T37</t>
+          <t xml:space="preserve">BLOCO 7</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Definir onde mora o custo estimado</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Decision</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PricebookEntry ou Product2</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nao ha campo de custo em Product2, PricebookEntry, Vehicle nem Asset. Definir onde mora e de onde vem antes de criar. Em Autos exonerados o custo e o do veiculo exonerado</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T01</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RN10</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">MARGEM E RASTREABILIDADE</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">T38</t>
+          <t xml:space="preserve">T37</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Campo de custo e campo de margem</t>
+          <t xml:space="preserve">Definir onde mora o custo estimado</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">CustomField</t>
+          <t xml:space="preserve">Decision</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Campo de custo no T37 e margem na linha</t>
+          <t xml:space="preserve">PricebookEntry ou Product2</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Criar o campo de custo definido no T37 e o campo de margem calculado sobre ele</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T37</t>
+          <t xml:space="preserve">Confirmado que nao ha campo de custo em Product2, PricebookEntry, Vehicle, Asset nem QuoteLineItem. Definir onde mora e de onde vem antes de criar. Em Autos exonerados o custo e o do veiculo exonerado</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -1689,34 +1669,39 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">CONFIRMADO, decidir</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">T39</t>
+          <t xml:space="preserve">T38</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Esconder custo e margem do assessor</t>
+          <t xml:space="preserve">Campo de custo e campo de margem</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">PermissionSet mais FLS</t>
+          <t xml:space="preserve">CustomField</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Campo de custo no T37 e margem na linha</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deixar custo e margem invisiveis ao assessor. A exibicao ao aprovador e da HU-065</t>
+          <t xml:space="preserve">Criar o campo de custo definido no T37 e o campo de margem calculado sobre ele</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t xml:space="preserve">T38</t>
+          <t xml:space="preserve">T37</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -1733,37 +1718,32 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">T40</t>
+          <t xml:space="preserve">T39</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Campos de rastreabilidade do desconto</t>
+          <t xml:space="preserve">Esconder custo e margem do assessor</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">CustomField</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QuoteLineItem: origem do desconto e regra aplicada</t>
+          <t xml:space="preserve">PermissionSet mais FLS</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registrar a origem, automatico ou manual, e a regra ou escalao que determinou o valor. Desconto e cashback registrados separados</t>
+          <t xml:space="preserve">Deixar custo e margem invisiveis ao assessor. A exibicao ao aprovador e da HU-065</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t xml:space="preserve">T14</t>
+          <t xml:space="preserve">T38</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN13</t>
+          <t xml:space="preserve">RN10</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -1775,37 +1755,37 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">T41</t>
+          <t xml:space="preserve">T40</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registrar as regras descartadas</t>
+          <t xml:space="preserve">Campos de rastreabilidade do desconto</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reuso</t>
+          <t xml:space="preserve">CustomField</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nebula Logger</t>
+          <t xml:space="preserve">QuoteLineItem: origem do desconto e regra aplicada</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registrar qual regra aplicou e quais foram descartadas no Nebula Logger, que ja esta instalado. Nao criar campo de log</t>
+          <t xml:space="preserve">Registrar a origem, automatico ou manual, e a regra ou escalao que determinou o valor. Desconto e cashback registrados separados</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t xml:space="preserve">T32</t>
+          <t xml:space="preserve">T14</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Escenarios 15 e 24</t>
+          <t xml:space="preserve">RN13</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -1817,61 +1797,66 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOCO 8</t>
+          <t xml:space="preserve">T41</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">FECHAMENTO</t>
+          <t xml:space="preserve">Registrar as regras descartadas</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reuso</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nebula Logger</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Registrar qual regra aplicou e quais foram descartadas no Nebula Logger, que ja esta instalado. Nao criar campo de log</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T32</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Escenarios 15 e 24</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A FAZER</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">T42</t>
+          <t xml:space="preserve">BLOCO 8</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reusar o processo de aprovacao ja ativo</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reuso</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DiscountApproval em Quote</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Partir do processo que ja esta ativo. Antes de redesenhar, levantar por que GQ_Discount_Approval e GQ_Discount_Approval_Chain em Opportunity ficaram obsoletos</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RN4, HU-065</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">FECHAMENTO</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">T43</t>
+          <t xml:space="preserve">T42</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reusar Aprobador_Config__mdt</t>
+          <t xml:space="preserve">Reusar o processo de aprovacao ja ativo</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1881,22 +1866,17 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aprobador_Config__mdt</t>
+          <t xml:space="preserve">DiscountApproval em Quote</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usar o metadata de aprovador que ja existe antes de criar outro</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T42</t>
+          <t xml:space="preserve">Partir do processo que ja esta ativo. Antes de redesenhar, levantar por que GQ_Discount_Approval e GQ_Discount_Approval_Chain em Opportunity ficaram obsoletos</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-065</t>
+          <t xml:space="preserve">RN4, HU-065</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -1908,32 +1888,37 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">T44</t>
+          <t xml:space="preserve">T43</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trigger Order nos flows criados</t>
+          <t xml:space="preserve">Reusar Aprobador_Config__mdt</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Object Manager</t>
+          <t xml:space="preserve">Reuso</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trigger Order de cada flow novo</t>
+          <t xml:space="preserve">Aprobador_Config__mdt</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Definir a Trigger Order em cada flow que esta HU criar em Quote e Order</t>
+          <t xml:space="preserve">Usar o metadata de aprovador que ja existe antes de criar outro</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T42</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Governanca</t>
+          <t xml:space="preserve">HU-065</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -1945,37 +1930,32 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">T45</t>
+          <t xml:space="preserve">T44</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Traduzir os rotulos para espanhol</t>
+          <t xml:space="preserve">Trigger Order nos flows criados</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Translation</t>
+          <t xml:space="preserve">Object Manager</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Translation Workbench</t>
+          <t xml:space="preserve">Trigger Order de cada flow novo</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Traduzir campos, valores de picklist e mensagens de alerta criados nesta HU</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T25</t>
+          <t xml:space="preserve">Definir a Trigger Order em cada flow que esta HU criar em Quote e Order</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Convencao GRPQM</t>
+          <t xml:space="preserve">Governanca</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -1987,40 +1967,82 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t xml:space="preserve">T45</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traduzir os rotulos para espanhol</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Translation</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Translation Workbench</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traduzir campos, valores de picklist e mensagens de alerta criados nesta HU</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T25</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Convencao GRPQM</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A FAZER</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t xml:space="preserve">T46</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t xml:space="preserve">Testes dos vinte e seis escenarios</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t xml:space="preserve">ApexClass</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t xml:space="preserve">Testes do procedure</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t xml:space="preserve">Cobrir os escenarios 1 a 26, com um caso por nivel da escala e um por sociedade</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t xml:space="preserve">T23, T32</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="G59" t="inlineStr">
         <is>
           <t xml:space="preserve">Todos</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="H59" t="inlineStr">
         <is>
           <t xml:space="preserve">A FAZER</t>
         </is>
@@ -2044,7 +2066,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-064 - Colunas padrao avaliadas antes de criar campo</t>
+          <t xml:space="preserve">HU-064 - Colunas padrao avaliadas antes de criar campo. Coluna Nota confirmada no describe de 18/08</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2227,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Calculado, UnitPrice vezes Quantity</t>
+          <t xml:space="preserve">somente leitura, UnitPrice vezes Quantity</t>
         </is>
       </c>
     </row>
@@ -2237,7 +2259,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Calculado</t>
+          <t xml:space="preserve">somente leitura</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2350,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivado das linhas e somente leitura. Nao recebe desconto de cabecalho</t>
+          <t xml:space="preserve">gravavel=false e criavel=false. E derivado das linhas e nao recebe escrita</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2382,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Calculado</t>
+          <t xml:space="preserve">calculado=true, somente leitura</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2414,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Calculado</t>
+          <t xml:space="preserve">calculado=true, somente leitura</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2446,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Calculado</t>
+          <t xml:space="preserve">somente leitura</t>
         </is>
       </c>
     </row>
@@ -2436,27 +2458,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Status</t>
+          <t xml:space="preserve">Tax</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Picklist</t>
+          <t xml:space="preserve">Currency</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Condicao requiere autorizacion, Escenario 2</t>
+          <t xml:space="preserve">Imposto do documento</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">AVALIAR PRIMEIRO</t>
+          <t xml:space="preserve">REUSAR</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ver no T01 se ja ha valor que sirva antes de criar campo</t>
+          <t xml:space="preserve">gravavel=true. Coluna padrao livre, serve tambem a HU-105</t>
         </is>
       </c>
     </row>
@@ -2468,22 +2490,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">ExpirationDate</t>
+          <t xml:space="preserve">Status</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Date</t>
+          <t xml:space="preserve">Picklist</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia do documento</t>
+          <t xml:space="preserve">Condicao requiere autorizacion, Escenario 2</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">REUSAR</t>
+          <t xml:space="preserve">AVALIAR, VER T22</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NAO restrita. Ja tem Draft, Approved, Rejected, Accepted, Denied, Pendiente, Pedido futuro e En transito</t>
         </is>
       </c>
     </row>
@@ -2495,17 +2522,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pricebook2Id</t>
+          <t xml:space="preserve">ExpirationDate</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lookup</t>
+          <t xml:space="preserve">Date</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lista de precos vigente, premissa da HU-038</t>
+          <t xml:space="preserve">Vigencia do documento</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2517,22 +2544,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">OrderItem</t>
+          <t xml:space="preserve">Quote</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">UnitPrice</t>
+          <t xml:space="preserve">Pricebook2Id</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Currency</t>
+          <t xml:space="preserve">Lookup</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preco da linha do pedido</t>
+          <t xml:space="preserve">Lista de precos vigente, premissa da HU-038</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -2549,7 +2576,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ListPrice</t>
+          <t xml:space="preserve">UnitPrice</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2559,17 +2586,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precio de Lista da linha do pedido</t>
+          <t xml:space="preserve">Preco da linha do pedido</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
           <t xml:space="preserve">REUSAR</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Somente leitura</t>
         </is>
       </c>
     </row>
@@ -2581,7 +2603,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">TotalPrice</t>
+          <t xml:space="preserve">ListPrice</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2591,12 +2613,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Total da linha do pedido</t>
+          <t xml:space="preserve">Precio de Lista da linha do pedido</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
           <t xml:space="preserve">REUSAR</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Somente leitura</t>
         </is>
       </c>
     </row>
@@ -2608,34 +2635,39 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Discount</t>
+          <t xml:space="preserve">TotalPrice</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Currency</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Percentual de desconto no pedido, Escenario 17</t>
+          <t xml:space="preserve">Total da linha do pedido</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAO EXISTE, CRIAR</t>
+          <t xml:space="preserve">REUSAR</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirmar no T01. E a unica coluna de desconto que falta de verdade</t>
+          <t xml:space="preserve">somente leitura</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Order</t>
+          <t xml:space="preserve">OrderItem</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">TotalAmount</t>
+          <t xml:space="preserve">TotalLineAmount</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2645,7 +2677,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Total do pedido</t>
+          <t xml:space="preserve">Total da linha ja com desconto, Escenario 17</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2655,46 +2687,46 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Calculado</t>
+          <t xml:space="preserve">gravavel=true. O VALOR do desconto cabe aqui, so o percentual e que nao</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Order</t>
+          <t xml:space="preserve">OrderItem</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Status</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Picklist</t>
+          <t xml:space="preserve">Discount</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Estado do pedido</t>
+          <t xml:space="preserve">Percentual de desconto no pedido, Escenario 17</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">REUSAR</t>
+          <t xml:space="preserve">NAO EXISTE, CRIAR</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmado no describe. E a unica coluna de desconto que falta de verdade</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">PricebookEntry</t>
+          <t xml:space="preserve">Order</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">PrecioMinimoAsesor__c</t>
+          <t xml:space="preserve">TotalAmount</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2704,7 +2736,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Base de calculo da escala, RN5</t>
+          <t xml:space="preserve">Total do pedido</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2714,61 +2746,56 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ja existe na org</t>
+          <t xml:space="preserve">Calculado</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">PricebookEntry</t>
+          <t xml:space="preserve">Order</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">PrecioExoneradoMinimo__c</t>
+          <t xml:space="preserve">Status</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Currency</t>
+          <t xml:space="preserve">Picklist</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Base de calculo exonerada, RN5</t>
+          <t xml:space="preserve">Estado do pedido</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
           <t xml:space="preserve">REUSAR</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ja existe na org</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">PricebookEntry</t>
+          <t xml:space="preserve">Order</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">PrecioExonerado__c</t>
+          <t xml:space="preserve">StatusCode</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Currency</t>
+          <t xml:space="preserve">Picklist</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preco exonerado</t>
+          <t xml:space="preserve">Estado interno do pedido</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2778,7 +2805,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ja existe na org</t>
+          <t xml:space="preserve">gravavel=true, criavel=false</t>
         </is>
       </c>
     </row>
@@ -2790,7 +2817,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastos__c</t>
+          <t xml:space="preserve">PrecioMinimoAsesor__c</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2800,7 +2827,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastos da entrada de preco</t>
+          <t xml:space="preserve">Base de calculo da escala, RN5</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2822,17 +2849,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">AplicaCashback__c</t>
+          <t xml:space="preserve">PrecioExoneradoMinimo__c</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Checkbox</t>
+          <t xml:space="preserve">Currency</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bandeira de cashback, RN11</t>
+          <t xml:space="preserve">Base de calculo exonerada, RN5</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2854,7 +2881,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">MontoCashback__c</t>
+          <t xml:space="preserve">PrecioExonerado__c</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2864,7 +2891,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Montante de cashback, RN11</t>
+          <t xml:space="preserve">Preco exonerado</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2886,17 +2913,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">VigenciaDesde__c</t>
+          <t xml:space="preserve">Gastos__c</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Date</t>
+          <t xml:space="preserve">Currency</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vigencia do cashback, RN11</t>
+          <t xml:space="preserve">Gastos da entrada de preco</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2918,44 +2945,49 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">UnitPrice</t>
+          <t xml:space="preserve">AplicaCashback__c</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Currency</t>
+          <t xml:space="preserve">Checkbox</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precio de Lista</t>
+          <t xml:space="preserve">Bandeira de cashback, RN11</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
           <t xml:space="preserve">REUSAR</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ja existe na org</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product2</t>
+          <t xml:space="preserve">PricebookEntry</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">BusinessBrandId</t>
+          <t xml:space="preserve">MontoCashback__c</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lookup</t>
+          <t xml:space="preserve">Currency</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marca, chave da escala da RN5</t>
+          <t xml:space="preserve">Montante de cashback, RN11</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2965,56 +2997,61 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Padrao do Automotive. BusinessBrand tem 23 registros</t>
+          <t xml:space="preserve">Ja existe na org</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product2</t>
+          <t xml:space="preserve">PricebookEntry</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Family</t>
+          <t xml:space="preserve">VigenciaDesde__c</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Picklist</t>
+          <t xml:space="preserve">Date</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Familia, criterio de Repuestos</t>
+          <t xml:space="preserve">Vigencia do cashback, RN11</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
           <t xml:space="preserve">REUSAR</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ja existe na org</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product2</t>
+          <t xml:space="preserve">PricebookEntry</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">ProductCode</t>
+          <t xml:space="preserve">UnitPrice</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text</t>
+          <t xml:space="preserve">Currency</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">SKU, criterio de Repuestos</t>
+          <t xml:space="preserve">Precio de Lista</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3026,17 +3063,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleDefinition</t>
+          <t xml:space="preserve">Product2</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">(objeto)</t>
+          <t xml:space="preserve">BusinessBrandId</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lookup</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modelo, chave da escala da RN5</t>
+          <t xml:space="preserve">Marca, chave da escala da RN5</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3046,78 +3088,78 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">229 registros na org</t>
+          <t xml:space="preserve">Padrao do Automotive. BusinessBrand tem 23 registros</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">BusinessBrand</t>
+          <t xml:space="preserve">Product2</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">(objeto)</t>
+          <t xml:space="preserve">Family</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Picklist</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marca, chave da escala da RN5</t>
+          <t xml:space="preserve">Familia, criterio de Repuestos</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
           <t xml:space="preserve">REUSAR</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23 registros na org</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">UserRole</t>
+          <t xml:space="preserve">Product2</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">(objeto)</t>
+          <t xml:space="preserve">ProductCode</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nivel do usuario, RN4 e RN5</t>
+          <t xml:space="preserve">SKU, criterio de Repuestos</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">REUSAR PARCIAL</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tem Gerente de Marca e Director. Falta Gerente de Ventas e Vicepresidencia</t>
+          <t xml:space="preserve">REUSAR</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sociedad_Config__mdt</t>
+          <t xml:space="preserve">VehicleDefinition</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">(metadata)</t>
+          <t xml:space="preserve">(objeto)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sociedade, chave da escala</t>
+          <t xml:space="preserve">Modelo, chave da escala da RN5</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3127,105 +3169,105 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">14 registros na org</t>
+          <t xml:space="preserve">229 registros na org</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quote</t>
+          <t xml:space="preserve">BusinessBrand</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">(campo de cashback)</t>
+          <t xml:space="preserve">(objeto)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Montante destinado a cashback, RN11</t>
+          <t xml:space="preserve">Marca, chave da escala da RN5</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAO EXISTE, CRIAR</t>
+          <t xml:space="preserve">REUSAR</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sem coluna padrao equivalente</t>
+          <t xml:space="preserve">23 registros na org</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">QuoteLineItem</t>
+          <t xml:space="preserve">UserRole</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">(origem do desconto)</t>
+          <t xml:space="preserve">(objeto)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automatico ou manual, RN13</t>
+          <t xml:space="preserve">Nivel do usuario, RN4 e RN5</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAO EXISTE, CRIAR</t>
+          <t xml:space="preserve">REUSAR PARCIAL</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sem coluna padrao equivalente</t>
+          <t xml:space="preserve">Tem Gerente de Marca e Director. Falta Gerente de Ventas e Vicepresidencia</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">QuoteLineItem</t>
+          <t xml:space="preserve">Sociedad_Config__mdt</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">(regra aplicada)</t>
+          <t xml:space="preserve">(metadata)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Regra ou escalao que determinou, RN13</t>
+          <t xml:space="preserve">Sociedade, chave da escala</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAO EXISTE, CRIAR</t>
+          <t xml:space="preserve">REUSAR</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sem coluna padrao equivalente</t>
+          <t xml:space="preserve">14 registros na org</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product2 ou PricebookEntry</t>
+          <t xml:space="preserve">Quote</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">(custo estimado)</t>
+          <t xml:space="preserve">(campo de cashback)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Base da margem, RN10</t>
+          <t xml:space="preserve">Montante destinado a cashback, RN11</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3235,7 +3277,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nenhum campo de custo em Product2, PricebookEntry, Vehicle nem Asset</t>
+          <t xml:space="preserve">Sem coluna padrao equivalente</t>
         </is>
       </c>
     </row>
@@ -3247,20 +3289,101 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t xml:space="preserve">(origem do desconto)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Automatico ou manual, RN13</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NAO EXISTE, CRIAR</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sem coluna padrao equivalente</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QuoteLineItem</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(regra aplicada)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regra ou escalao que determinou, RN13</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NAO EXISTE, CRIAR</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sem coluna padrao equivalente</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product2 ou PricebookEntry</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(custo estimado)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Base da margem, RN10</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NAO EXISTE, CRIAR</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmado: nenhum campo de custo em Product2, PricebookEntry, Vehicle, Asset nem QuoteLineItem</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QuoteLineItem</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
           <t xml:space="preserve">(margem)</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t xml:space="preserve">Margem resultante, RN10</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t xml:space="preserve">NAO EXISTE, CRIAR</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t xml:space="preserve">Precisa de FLS para esconder do assessor</t>
         </is>

</xml_diff>